<commit_message>
Event link extraction, token usage output
</commit_message>
<xml_diff>
--- a/events_output_test.xlsx
+++ b/events_output_test.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Rejected Events" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Already on Calendar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -134,9 +133,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K7" headerRowCount="1">
-  <autoFilter ref="A1:K7"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:L6" headerRowCount="1">
+  <autoFilter ref="A1:L6"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Event Title"/>
     <tableColumn id="2" name="Fit Score"/>
     <tableColumn id="3" name="Confidence"/>
@@ -145,18 +144,19 @@
     <tableColumn id="6" name="URL"/>
     <tableColumn id="7" name="Start Time"/>
     <tableColumn id="8" name="Location"/>
-    <tableColumn id="9" name="Status"/>
-    <tableColumn id="10" name="Description"/>
-    <tableColumn id="11" name="Fit Reason"/>
+    <tableColumn id="9" name="Signup Link"/>
+    <tableColumn id="10" name="Status"/>
+    <tableColumn id="11" name="Description"/>
+    <tableColumn id="12" name="Fit Reason"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K6" headerRowCount="1">
-  <autoFilter ref="A1:K6"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:L10" headerRowCount="1">
+  <autoFilter ref="A1:L10"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Event Title"/>
     <tableColumn id="2" name="Fit Score"/>
     <tableColumn id="3" name="Confidence"/>
@@ -165,9 +165,10 @@
     <tableColumn id="6" name="URL"/>
     <tableColumn id="7" name="Start Time"/>
     <tableColumn id="8" name="Location"/>
-    <tableColumn id="9" name="Status"/>
-    <tableColumn id="10" name="Description"/>
-    <tableColumn id="11" name="Fit Reason"/>
+    <tableColumn id="9" name="Signup Link"/>
+    <tableColumn id="10" name="Status"/>
+    <tableColumn id="11" name="Description"/>
+    <tableColumn id="12" name="Fit Reason"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
 </table>
@@ -462,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -472,10 +473,11 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,15 +523,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Signup Link</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Fit Reason</t>
         </is>
@@ -538,294 +545,270 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>From prototype to production with Kiro &amp; Kiro CLI</t>
+          <t>SCL Course: Machine Learning Applications for Supply Chain Planning (Virtual/Instructor-Lead)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46212</v>
+        <v>46279</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://ai.gatech.edu/events</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6:00 PM EDT</t>
+          <t>1:00 PM EDT</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Virtual/Instructor-led</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>https://ai.gatech.edu/event/scl-course-machine-learning-applications-supply-chain-planning-virtualinstructor-lead</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>The event title and description contain no mention of AI, machine learning, or automation, triggering the automatic 1 rating regardless of Georgia focus or other factors.</t>
+          <t>Apply machine learning with Python and Power BI to optimize supply chain forecasting, inventory, and maintenance.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with clear machine learning content hosted by Georgia Tech (a Georgia institution), which qualifies it for a mid-to-high score despite not being in-person.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Using Generative AI on Structured Data</t>
+          <t>SCL Course: Generative AI Application for Supply Chain Professionals (Virtual/Instructor-led)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46209</v>
+        <v>46496</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://ai.gatech.edu/events</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6:30 PM EDT</t>
+          <t>8:00 PM EDT</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Virtual/Instructor-led</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>https://ai.gatech.edu/event/scl-course-generative-ai-application-supply-chain-professionals-virtualinstructor-led-0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Virtual-only event with clear AI content (generative AI on structured data) but no Georgia focus or host organization information provided, and minimal event details available.</t>
+          <t>Participants will explore generative AI fundamentals, prompt engineering, and practical applications such as automated inventory systems, predictive maintenance, and route optimization.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event with strong AI content (generative AI, prompt engineering, applications) hosted by Georgia Tech institution scores highly despite not being in-person.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>How to Use AI for Academic Research</t>
+          <t>SCL Course: Generative AI Application for Supply Chain Professionals (Onsite/In-Person)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46214</v>
+        <v>46678</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://ai.gatech.edu/events</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9:00 AM EDT</t>
+          <t>8:00 PM EDT</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Georgia Tech Savannah</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>https://ai.gatech.edu/event/scl-course-generative-ai-application-supply-chain-professionals-onsitein-person</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Virtual-only event with clear AI content (academic research applications) but no Georgia focus or hosting institution mentioned, and minimal event details provided.</t>
+          <t>Participants will explore generative AI fundamentals, prompt engineering, and practical applications such as automated inventory systems, predictive maintenance, and route optimization.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>In-person Georgia Tech event with substantial AI content (generative AI fundamentals, prompt engineering, supply chain applications) that is educational rather than a sales pitch.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AWS: Build Resilient Multi-Step Applications With Just Code</t>
+          <t>Manufacturing Technology Challenges: Practical Solutions for Today's Pla...</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46219</v>
+        <v>46239</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
+          <t>11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/tech-educational-panel</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Virtual AWS technical event with AI/automation relevance (multi-step applications, resilient systems) hosted for Georgia audience, though short description limits confidence in AI content depth.</t>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>The event description is empty with no mention of AI, machine learning, or automation in the title or available details, making it an automatic 1 despite the Georgia-based organization.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FREE REMOTE | LADIES IN AI - We Learn. We Share. We Laugh.</t>
+          <t>AIMST - AI Conference - GMA Special Exhibitor and Moderator</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46219</v>
+        <v>46252</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>7:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/aimst---ai-conference---gma-special-exhibitor-and-moderator</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Event has clear AI focus ('Ladies in AI') and is free/educational, but lacks location specificity, Georgia connection, and detailed description to assess whether it's a Georgia-focused or Georgia-hosted virtual event versus a generic national event.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GA AI Alliance Networking Lunch</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>46234</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>July 5, 2026</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>11:45 AM EDT</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>In-person Georgia event with AI-relevant organization (GA AI Alliance) but minimal description prevents higher rating; networking lunch format suggests social rather than educational content.</t>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>AIMST is a known AI conference (strong fit for AI content), marked as in-person which scores highest, and hosted/promoted by Georgia Manufacturing Alliance suggesting Georgia relevance, though missing specific location details and event description reduce confidence slightly.</t>
         </is>
       </c>
     </row>
@@ -843,20 +826,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -902,15 +886,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Signup Link</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Fit Reason</t>
         </is>
@@ -919,7 +908,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Find a Startup to Help or Join</t>
+          <t>Coffee and Connections - Atlanta 7-16-2026</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -935,40 +924,45 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6:00 PM EDT</t>
+          <t>8:30 AM EDT</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/coffee-and-connections---atlanta-7-16-2026</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of other factors.</t>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Atlanta Tech Meet-Up</t>
+          <t>Networking Luncheon - Atlanta 7-16-2026</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -980,44 +974,49 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46210</v>
+        <v>46219</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6:00 PM EDT</t>
+          <t>11:30 AM EDT</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/networking-luncheon---atlanta-7-16-2026</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or other factors.</t>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Python Atlanta Meetup (In Person!)</t>
+          <t>WGMA Paint the Town- The Davis Companies</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1029,44 +1028,45 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46212</v>
+        <v>46225</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
+          <t>11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/wgma-paint-the-town--the-davis-companies</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Georgia location.</t>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, triggering an automatic score of 1 regardless of other factors.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Open House!</t>
+          <t>Murray Plastics Factory Tour - SMTA Joint Event - Gainesville</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1078,44 +1078,49 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46217</v>
+        <v>46233</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7:30 PM EDT</t>
+          <t>9:00 AM EDT</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Gainesville</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/murray-plastics-factory-tour---smta-joint-event---gainesville</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering automatic score of 1 per criteria.</t>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bytes &amp; Bites @ Krog St Market</t>
+          <t>Murray Plastics Factory Tour - SMTA Joint Event - Gainesville - AFTERNOON</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1127,37 +1132,250 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46227</v>
+        <v>46233</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>July 5, 2026</t>
+          <t>July 9, 2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11:45 AM EDT</t>
+          <t>11:30 AM EDT</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Krog St Market</t>
+          <t>Gainesville</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/murray-plastics-factory-tour---smta-joint-event---gainesville---afternoon</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Georgia location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Women of GMA Virtual Networking Event 8/11/26</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>July 9, 2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-81126</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Coffee and Connections - Atlanta 8-20-2026</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>July 9, 2026</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>8:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/coffee-and-connections-atlanta-8-20-2026</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or in-person format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Networking Luncheon - Atlanta 8-20-2026</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>July 9, 2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>11:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/networking-luncheon-atlanta-8-20-2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026 Georgia Manufacturing Summit</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>July 9, 2026</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>7:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/2026-georgia-manufacturing-summit</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available description contain zero mention of AI, machine learning, or automation, triggering the automatic 1 rating regardless of location or in-person status.</t>
         </is>
       </c>
     </row>
@@ -1167,88 +1385,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Event Title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Fit Score</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Confidence</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Event Date</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Date Scraped</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Fit Reason</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Token input/output optimization, iframe capture, load more extraction, pre scoring existing event check
</commit_message>
<xml_diff>
--- a/events_output_test.xlsx
+++ b/events_output_test.xlsx
@@ -472,7 +472,7 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
@@ -596,7 +596,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Virtual-only event with clear machine learning content hosted by Georgia Tech (a Georgia institution), which qualifies it for a mid-to-high score despite not being in-person.</t>
+          <t>Virtual event with clear ML/AI content hosted by Georgia Tech (a Georgia institution), scoring above the typical virtual event baseline, but not reaching higher tiers since it's not in-person and appears to be a paid training course rather than a broader educational discussion.</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Virtual event with strong AI content (generative AI, prompt engineering, applications) hosted by Georgia Tech institution scores highly despite not being in-person.</t>
+          <t>Virtual event hosted by Georgia Tech (a Georgia institution) with strong AI content covering generative AI fundamentals and practical supply chain applications, scoring 3-4 per Georgia Tech virtual event criteria, elevated to 4 for substantive technical focus.</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -712,7 +712,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>In-person Georgia Tech event with substantial AI content (generative AI fundamentals, prompt engineering, supply chain applications) that is educational rather than a sales pitch.</t>
+          <t>In-person Georgia Tech event with strong AI content (generative AI, prompt engineering, practical applications), though it appears to be a paid training course rather than a purely educational conference.</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>11:00 AM EDT</t>
+          <t>11:00 AM - 1:30 PM EDT</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -762,7 +762,7 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>The event description is empty with no mention of AI, machine learning, or automation in the title or available details, making it an automatic 1 despite the Georgia-based organization.</t>
+          <t>The event description is empty with no mention of AI, machine learning, or automation in the title or available details, making it an automatic 1 per criteria despite the Georgia-based organization.</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>AIMST is a known AI conference (strong fit for AI content), marked as in-person which scores highest, and hosted/promoted by Georgia Manufacturing Alliance suggesting Georgia relevance, though missing specific location details and event description reduce confidence slightly.</t>
+          <t>AIMST is a known AI conference with in-person format, Georgia connection through GMA signup link, and clear AI focus, but minimal description details reduce confidence slightly.</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
@@ -934,7 +934,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8:30 AM EDT</t>
+          <t>8:30 AM - 10:00 AM EDT</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -955,7 +955,7 @@
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of in-person Atlanta location.</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11:30 AM EDT</t>
+          <t>11:30 AM - 1:00 PM EDT</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1009,7 +1009,7 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>11:00 AM EDT</t>
+          <t>11:00 AM - 1:00 PM EDT</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -1059,7 +1059,7 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, triggering an automatic score of 1 regardless of other factors.</t>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering an automatic 1 score regardless of other criteria.</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9:00 AM EDT</t>
+          <t>9:00 AM - 12:00 PM EDT</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1113,7 +1113,7 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or other factors.</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11:30 AM EDT</t>
+          <t>11:30 AM - 4:00 PM EDT</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1167,7 +1167,7 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Georgia location.</t>
+          <t>The event is a factory tour with zero mention of AI, machine learning, or automation in the title or description, making it an automatic 1 regardless of location.</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3:30 PM EDT</t>
+          <t>3:30 PM - 4:30 PM EDT</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1217,7 +1217,7 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of other factors.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8:30 AM EDT</t>
+          <t>8:30 AM - 10:00 AM EDT</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1271,7 +1271,7 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or in-person format.</t>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Atlanta location.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11:30 AM EDT</t>
+          <t>11:30 AM - 1:00 PM EDT</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1325,7 +1325,7 @@
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
+          <t>The event is a generic networking luncheon with zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7:00 AM EDT</t>
+          <t>7:00 AM - 4:00 PM EDT</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1375,7 +1375,7 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>The event title and available description contain zero mention of AI, machine learning, or automation, triggering the automatic 1 rating regardless of location or in-person status.</t>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or other criteria.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reduced # of links being sent to AI input
</commit_message>
<xml_diff>
--- a/events_output_test.xlsx
+++ b/events_output_test.xlsx
@@ -133,8 +133,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:L6" headerRowCount="1">
-  <autoFilter ref="A1:L6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:L7" headerRowCount="1">
+  <autoFilter ref="A1:L7"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Event Title"/>
     <tableColumn id="2" name="Fit Score"/>
@@ -154,8 +154,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:L10" headerRowCount="1">
-  <autoFilter ref="A1:L10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:L9" headerRowCount="1">
+  <autoFilter ref="A1:L9"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Event Title"/>
     <tableColumn id="2" name="Fit Score"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Virtual event with clear ML/AI content hosted by Georgia Tech (a Georgia institution), scoring above the typical virtual event baseline, but not reaching higher tiers since it's not in-person and appears to be a paid training course rather than a broader educational discussion.</t>
+          <t>Virtual event with strong AI/ML content (machine learning applications) hosted by Georgia Tech, a Georgia institution, which elevates it above the typical virtual-only score.</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Virtual event hosted by Georgia Tech (a Georgia institution) with strong AI content covering generative AI fundamentals and practical supply chain applications, scoring 3-4 per Georgia Tech virtual event criteria, elevated to 4 for substantive technical focus.</t>
+          <t>Virtual event hosted by Georgia Tech with substantive AI content (generative AI fundamentals, prompt engineering, practical supply chain applications), meeting the criteria for Georgia institution-hosted virtual events scoring 3-4.</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>In-person Georgia Tech event with strong AI content (generative AI, prompt engineering, practical applications), though it appears to be a paid training course rather than a purely educational conference.</t>
+          <t>In-person Georgia Tech event with substantive AI content (generative AI, prompt engineering, supply chain applications) that appears educational rather than a sales pitch.</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>The event description is empty with no mention of AI, machine learning, or automation in the title or available details, making it an automatic 1 per criteria despite the Georgia-based organization.</t>
+          <t>The event title and description contain zero explicit mention of AI, machine learning, or automation, making it an automatic 1 regardless of other criteria.</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,57 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>AIMST is a known AI conference with in-person format, Georgia connection through GMA signup link, and clear AI focus, but minimal description details reduce confidence slightly.</t>
+          <t>AIMST is a known AI conference with in-person format, hosted by Georgia Manufacturing Alliance (Georgia-focused organization), and explicitly mentions AI in the title, though the missing location field and empty description reduce confidence slightly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026 Georgia Manufacturing Summit</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>July 9, 2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>7:00 AM - 4:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/2026-georgia-manufacturing-summit</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or available description, making it an automatic 1 regardless of location.</t>
         </is>
       </c>
     </row>
@@ -826,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -955,7 +1005,7 @@
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of in-person Atlanta location.</t>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1059,7 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
+          <t>Event is a generic networking luncheon with zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Atlanta location.</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1109,7 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering an automatic 1 score regardless of other criteria.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of other factors.</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1163,7 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or other factors.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or in-person status.</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1217,7 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>The event is a factory tour with zero mention of AI, machine learning, or automation in the title or description, making it an automatic 1 regardless of location.</t>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Georgia location.</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1267,7 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of other factors.</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1321,7 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Atlanta location.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
         </is>
       </c>
     </row>
@@ -1325,57 +1375,7 @@
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>The event is a generic networking luncheon with zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026 Georgia Manufacturing Summit</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>46280</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>July 9, 2026</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://www.georgiamanufacturingalliance.com/events/</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>7:00 AM - 4:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>https://www.georgiamanufacturingalliance.com/events/2026-georgia-manufacturing-summit</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or other criteria.</t>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of being in-person in Atlanta.</t>
         </is>
       </c>
     </row>

</xml_diff>